<commit_message>
CppPractice with L1 = 2, L2 = 4, L3 = 1, L4 = 0
</commit_message>
<xml_diff>
--- a/Practice_Bank.xlsx
+++ b/Practice_Bank.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20361"/>
   <workbookPr filterPrivacy="1" hidePivotFieldList="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F746996-0969-4303-8691-90B90EF0764A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11D67EBA-A5C8-4E6E-B55C-C84B31D34465}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="123">
   <si>
     <t>Basics</t>
   </si>
@@ -163,9 +163,6 @@
     <t>Program_Name</t>
   </si>
   <si>
-    <t>Hello World</t>
-  </si>
-  <si>
     <t>Time_Min</t>
   </si>
   <si>
@@ -370,16 +367,34 @@
     <t>শীট ১: Problems (মূল শীট)</t>
   </si>
   <si>
-    <t>My Name</t>
-  </si>
-  <si>
-    <t>Bio Data</t>
-  </si>
-  <si>
-    <t>Sum of 2</t>
-  </si>
-  <si>
     <t>Average 3</t>
+  </si>
+  <si>
+    <t>A Complete Guide to Programming in C++</t>
+  </si>
+  <si>
+    <t>Do</t>
+  </si>
+  <si>
+    <t>01_Arithmetic</t>
+  </si>
+  <si>
+    <t>Using with if else</t>
+  </si>
+  <si>
+    <t>01_If_Basic</t>
+  </si>
+  <si>
+    <t>01_Hello</t>
+  </si>
+  <si>
+    <t>02_MyName</t>
+  </si>
+  <si>
+    <t>03_BioData</t>
+  </si>
+  <si>
+    <t>04_Sum</t>
   </si>
 </sst>
 </file>
@@ -551,7 +566,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -657,6 +672,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -978,34 +994,34 @@
   <sheetData>
     <row r="1" spans="2:5" ht="23.25" customHeight="1">
       <c r="B1" s="32" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="2" spans="2:5" ht="15.75" thickBot="1"/>
     <row r="3" spans="2:5" s="18" customFormat="1" ht="20.25" customHeight="1">
       <c r="B3" s="16" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C3" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="D3" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="D3" s="19" t="s">
-        <v>59</v>
-      </c>
       <c r="E3" s="20" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" spans="2:5" ht="15.75">
       <c r="B4" s="9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C4" s="10">
         <f ca="1">TODAY()</f>
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E4" s="21">
         <f>COUNTIF(Problems!D:D,"L1 (Copy)")</f>
@@ -1014,30 +1030,30 @@
     </row>
     <row r="5" spans="2:5" ht="15.75">
       <c r="B5" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C5" s="11">
         <f>COUNTA(Problems!E:E)-1</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E5" s="21">
         <f>COUNTIF(Problems!D:D,"L2 (Modify)")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="2:5" ht="15.75">
       <c r="B6" s="9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C6" s="11">
         <f>COUNTIF(Problems!H:H,"✅ Done")</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E6" s="21">
         <f>COUNTIF(Problems!D:D,"L3 (Combine)")</f>
@@ -1046,14 +1062,14 @@
     </row>
     <row r="7" spans="2:5" ht="16.5" thickBot="1">
       <c r="B7" s="9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C7" s="11">
         <f>COUNTIF(Problems!H:H, "⏳ In Progress")</f>
         <v>0</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E7" s="22">
         <f>COUNTIF(Problems!D:D,"L4 (Create)")</f>
@@ -1062,56 +1078,56 @@
     </row>
     <row r="8" spans="2:5" ht="15.75">
       <c r="B8" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C8" s="11">
         <f>COUNTIF(Problems!H:H, "⬜ Not Started")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="2:5" ht="15.75">
       <c r="B9" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C9" s="11">
         <f>SUM(Problems!G:G)/60</f>
-        <v>0</v>
+        <v>1.3333333333333333</v>
       </c>
     </row>
     <row r="10" spans="2:5" ht="15.75">
       <c r="B10" s="9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C10" s="11">
         <f ca="1">COUNTIF(Problems!B:B,TODAY())</f>
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="2:5" ht="15.75">
       <c r="B11" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C11" s="11">
         <f ca="1">COUNTIFS(Problems!B:B,"&gt;="&amp;TODAY()-7,Problems!H:H,"✅ Done")/7</f>
-        <v>0</v>
+        <v>0.8571428571428571</v>
       </c>
     </row>
     <row r="12" spans="2:5" ht="16.5" thickBot="1">
       <c r="B12" s="12" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C12" s="13">
         <f>IFERROR(COUNTIF(Problems!H:H,"✅ Done")/COUNTA(Problems!E:E),0)</f>
-        <v>0</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="13" spans="2:5" ht="15.75" thickBot="1"/>
     <row r="14" spans="2:5" ht="15.75">
       <c r="B14" s="16" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C14" s="44" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D14" s="23"/>
       <c r="E14" s="24"/>
@@ -1121,13 +1137,13 @@
         <v>11</v>
       </c>
       <c r="C15" s="26" t="s">
+        <v>74</v>
+      </c>
+      <c r="D15" s="26" t="s">
         <v>75</v>
       </c>
-      <c r="D15" s="26" t="s">
+      <c r="E15" s="27" t="s">
         <v>76</v>
-      </c>
-      <c r="E15" s="27" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="16" spans="2:5">
@@ -1140,11 +1156,11 @@
       </c>
       <c r="D16" s="29">
         <f>SUMIF(Problems!$C:$C,B16,Problems!$G:$G)</f>
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="E16" s="7">
         <f>IFERROR(COUNTIFS(Problems!$C:$C,B16,Problems!$H:$H,"✅ Done")/COUNTIF(Problems!$C:$C,B16),0)</f>
-        <v>0</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="17" spans="2:5">
@@ -1153,15 +1169,15 @@
       </c>
       <c r="C17" s="29">
         <f>COUNTIF(Problems!$C:$C,B17)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D17" s="29">
         <f>SUMIF(Problems!$C:$C,B17,Problems!$G:$G)</f>
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E17" s="7">
         <f>IFERROR(COUNTIFS(Problems!$C:$C,B17,Problems!$H:$H,"✅ Done")/COUNTIF(Problems!$C:$C,B17),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="2:5">
@@ -1170,15 +1186,15 @@
       </c>
       <c r="C18" s="29">
         <f>COUNTIF(Problems!$C:$C,B18)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D18" s="29">
         <f>SUMIF(Problems!$C:$C,B18,Problems!$G:$G)</f>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="E18" s="7">
         <f>IFERROR(COUNTIFS(Problems!$C:$C,B18,Problems!$H:$H,"✅ Done")/COUNTIF(Problems!$C:$C,B18),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="2:5">
@@ -1324,16 +1340,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CF175F6-C32B-4A16-B92C-0C352068B40C}">
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J300"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
+    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="6" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="27" customHeight="1">
       <c r="B1" s="32" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15.75">
@@ -1341,38 +1358,40 @@
         <v>43</v>
       </c>
       <c r="B3" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C3" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="D3" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="F3" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="G3" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="H3" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="I3" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="J3" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I3" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="J3" s="6" t="s">
-        <v>47</v>
-      </c>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="4"/>
+      <c r="A4" s="42">
+        <v>46301</v>
+      </c>
       <c r="B4" s="4" t="str">
         <f>TEXT(A4,"dddd")</f>
-        <v>Saturday</v>
+        <v>Tuesday</v>
       </c>
       <c r="C4" s="4"/>
       <c r="G4">
@@ -1381,52 +1400,914 @@
       </c>
     </row>
     <row r="5" spans="1:10">
-      <c r="A5" s="4"/>
+      <c r="A5" s="42"/>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
     </row>
     <row r="6" spans="1:10">
-      <c r="A6" s="4"/>
+      <c r="A6" s="42"/>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
     </row>
     <row r="7" spans="1:10">
-      <c r="A7" s="4"/>
+      <c r="A7" s="42"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
     </row>
     <row r="8" spans="1:10">
-      <c r="A8" s="4"/>
+      <c r="A8" s="42"/>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
     </row>
     <row r="9" spans="1:10">
-      <c r="A9" s="4"/>
+      <c r="A9" s="42"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
     </row>
     <row r="10" spans="1:10">
-      <c r="A10" s="4"/>
+      <c r="A10" s="42"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="4"/>
+      <c r="A11" s="42"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
     </row>
     <row r="12" spans="1:10">
-      <c r="A12" s="4"/>
+      <c r="A12" s="42"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="4"/>
+      <c r="A13" s="42"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
     </row>
+    <row r="14" spans="1:10">
+      <c r="A14" s="45"/>
+    </row>
+    <row r="15" spans="1:10">
+      <c r="A15" s="45"/>
+    </row>
+    <row r="16" spans="1:10">
+      <c r="A16" s="45"/>
+    </row>
+    <row r="17" spans="1:1">
+      <c r="A17" s="45"/>
+    </row>
+    <row r="18" spans="1:1">
+      <c r="A18" s="45"/>
+    </row>
+    <row r="19" spans="1:1">
+      <c r="A19" s="45"/>
+    </row>
+    <row r="20" spans="1:1">
+      <c r="A20" s="45"/>
+    </row>
+    <row r="21" spans="1:1">
+      <c r="A21" s="45"/>
+    </row>
+    <row r="22" spans="1:1">
+      <c r="A22" s="45"/>
+    </row>
+    <row r="23" spans="1:1">
+      <c r="A23" s="45"/>
+    </row>
+    <row r="24" spans="1:1">
+      <c r="A24" s="45"/>
+    </row>
+    <row r="25" spans="1:1">
+      <c r="A25" s="45"/>
+    </row>
+    <row r="26" spans="1:1">
+      <c r="A26" s="45"/>
+    </row>
+    <row r="27" spans="1:1">
+      <c r="A27" s="45"/>
+    </row>
+    <row r="28" spans="1:1">
+      <c r="A28" s="45"/>
+    </row>
+    <row r="29" spans="1:1">
+      <c r="A29" s="45"/>
+    </row>
+    <row r="30" spans="1:1">
+      <c r="A30" s="45"/>
+    </row>
+    <row r="31" spans="1:1">
+      <c r="A31" s="45"/>
+    </row>
+    <row r="32" spans="1:1">
+      <c r="A32" s="45"/>
+    </row>
+    <row r="33" spans="1:1">
+      <c r="A33" s="45"/>
+    </row>
+    <row r="34" spans="1:1">
+      <c r="A34" s="45"/>
+    </row>
+    <row r="35" spans="1:1">
+      <c r="A35" s="45"/>
+    </row>
+    <row r="36" spans="1:1">
+      <c r="A36" s="45"/>
+    </row>
+    <row r="37" spans="1:1">
+      <c r="A37" s="45"/>
+    </row>
+    <row r="38" spans="1:1">
+      <c r="A38" s="45"/>
+    </row>
+    <row r="39" spans="1:1">
+      <c r="A39" s="45"/>
+    </row>
+    <row r="40" spans="1:1">
+      <c r="A40" s="45"/>
+    </row>
+    <row r="41" spans="1:1">
+      <c r="A41" s="45"/>
+    </row>
+    <row r="42" spans="1:1">
+      <c r="A42" s="45"/>
+    </row>
+    <row r="43" spans="1:1">
+      <c r="A43" s="45"/>
+    </row>
+    <row r="44" spans="1:1">
+      <c r="A44" s="45"/>
+    </row>
+    <row r="45" spans="1:1">
+      <c r="A45" s="45"/>
+    </row>
+    <row r="46" spans="1:1">
+      <c r="A46" s="45"/>
+    </row>
+    <row r="47" spans="1:1">
+      <c r="A47" s="45"/>
+    </row>
+    <row r="48" spans="1:1">
+      <c r="A48" s="45"/>
+    </row>
+    <row r="49" spans="1:1">
+      <c r="A49" s="45"/>
+    </row>
+    <row r="50" spans="1:1">
+      <c r="A50" s="45"/>
+    </row>
+    <row r="51" spans="1:1">
+      <c r="A51" s="45"/>
+    </row>
+    <row r="52" spans="1:1">
+      <c r="A52" s="45"/>
+    </row>
+    <row r="53" spans="1:1">
+      <c r="A53" s="45"/>
+    </row>
+    <row r="54" spans="1:1">
+      <c r="A54" s="45"/>
+    </row>
+    <row r="55" spans="1:1">
+      <c r="A55" s="45"/>
+    </row>
+    <row r="56" spans="1:1">
+      <c r="A56" s="45"/>
+    </row>
+    <row r="57" spans="1:1">
+      <c r="A57" s="45"/>
+    </row>
+    <row r="58" spans="1:1">
+      <c r="A58" s="45"/>
+    </row>
+    <row r="59" spans="1:1">
+      <c r="A59" s="45"/>
+    </row>
+    <row r="60" spans="1:1">
+      <c r="A60" s="45"/>
+    </row>
+    <row r="61" spans="1:1">
+      <c r="A61" s="45"/>
+    </row>
+    <row r="62" spans="1:1">
+      <c r="A62" s="45"/>
+    </row>
+    <row r="63" spans="1:1">
+      <c r="A63" s="45"/>
+    </row>
+    <row r="64" spans="1:1">
+      <c r="A64" s="45"/>
+    </row>
+    <row r="65" spans="1:1">
+      <c r="A65" s="45"/>
+    </row>
+    <row r="66" spans="1:1">
+      <c r="A66" s="45"/>
+    </row>
+    <row r="67" spans="1:1">
+      <c r="A67" s="45"/>
+    </row>
+    <row r="68" spans="1:1">
+      <c r="A68" s="45"/>
+    </row>
+    <row r="69" spans="1:1">
+      <c r="A69" s="45"/>
+    </row>
+    <row r="70" spans="1:1">
+      <c r="A70" s="45"/>
+    </row>
+    <row r="71" spans="1:1">
+      <c r="A71" s="45"/>
+    </row>
+    <row r="72" spans="1:1">
+      <c r="A72" s="45"/>
+    </row>
+    <row r="73" spans="1:1">
+      <c r="A73" s="45"/>
+    </row>
+    <row r="74" spans="1:1">
+      <c r="A74" s="45"/>
+    </row>
+    <row r="75" spans="1:1">
+      <c r="A75" s="45"/>
+    </row>
+    <row r="76" spans="1:1">
+      <c r="A76" s="45"/>
+    </row>
+    <row r="77" spans="1:1">
+      <c r="A77" s="45"/>
+    </row>
+    <row r="78" spans="1:1">
+      <c r="A78" s="45"/>
+    </row>
+    <row r="79" spans="1:1">
+      <c r="A79" s="45"/>
+    </row>
+    <row r="80" spans="1:1">
+      <c r="A80" s="45"/>
+    </row>
+    <row r="81" spans="1:1">
+      <c r="A81" s="45"/>
+    </row>
+    <row r="82" spans="1:1">
+      <c r="A82" s="45"/>
+    </row>
+    <row r="83" spans="1:1">
+      <c r="A83" s="45"/>
+    </row>
+    <row r="84" spans="1:1">
+      <c r="A84" s="45"/>
+    </row>
+    <row r="85" spans="1:1">
+      <c r="A85" s="45"/>
+    </row>
+    <row r="86" spans="1:1">
+      <c r="A86" s="45"/>
+    </row>
+    <row r="87" spans="1:1">
+      <c r="A87" s="45"/>
+    </row>
+    <row r="88" spans="1:1">
+      <c r="A88" s="45"/>
+    </row>
+    <row r="89" spans="1:1">
+      <c r="A89" s="45"/>
+    </row>
+    <row r="90" spans="1:1">
+      <c r="A90" s="45"/>
+    </row>
+    <row r="91" spans="1:1">
+      <c r="A91" s="45"/>
+    </row>
+    <row r="92" spans="1:1">
+      <c r="A92" s="45"/>
+    </row>
+    <row r="93" spans="1:1">
+      <c r="A93" s="45"/>
+    </row>
+    <row r="94" spans="1:1">
+      <c r="A94" s="45"/>
+    </row>
+    <row r="95" spans="1:1">
+      <c r="A95" s="45"/>
+    </row>
+    <row r="96" spans="1:1">
+      <c r="A96" s="45"/>
+    </row>
+    <row r="97" spans="1:1">
+      <c r="A97" s="45"/>
+    </row>
+    <row r="98" spans="1:1">
+      <c r="A98" s="45"/>
+    </row>
+    <row r="99" spans="1:1">
+      <c r="A99" s="45"/>
+    </row>
+    <row r="100" spans="1:1">
+      <c r="A100" s="45"/>
+    </row>
+    <row r="101" spans="1:1">
+      <c r="A101" s="45"/>
+    </row>
+    <row r="102" spans="1:1">
+      <c r="A102" s="45"/>
+    </row>
+    <row r="103" spans="1:1">
+      <c r="A103" s="45"/>
+    </row>
+    <row r="104" spans="1:1">
+      <c r="A104" s="45"/>
+    </row>
+    <row r="105" spans="1:1">
+      <c r="A105" s="45"/>
+    </row>
+    <row r="106" spans="1:1">
+      <c r="A106" s="45"/>
+    </row>
+    <row r="107" spans="1:1">
+      <c r="A107" s="45"/>
+    </row>
+    <row r="108" spans="1:1">
+      <c r="A108" s="45"/>
+    </row>
+    <row r="109" spans="1:1">
+      <c r="A109" s="45"/>
+    </row>
+    <row r="110" spans="1:1">
+      <c r="A110" s="45"/>
+    </row>
+    <row r="111" spans="1:1">
+      <c r="A111" s="45"/>
+    </row>
+    <row r="112" spans="1:1">
+      <c r="A112" s="45"/>
+    </row>
+    <row r="113" spans="1:1">
+      <c r="A113" s="45"/>
+    </row>
+    <row r="114" spans="1:1">
+      <c r="A114" s="45"/>
+    </row>
+    <row r="115" spans="1:1">
+      <c r="A115" s="45"/>
+    </row>
+    <row r="116" spans="1:1">
+      <c r="A116" s="45"/>
+    </row>
+    <row r="117" spans="1:1">
+      <c r="A117" s="45"/>
+    </row>
+    <row r="118" spans="1:1">
+      <c r="A118" s="45"/>
+    </row>
+    <row r="119" spans="1:1">
+      <c r="A119" s="45"/>
+    </row>
+    <row r="120" spans="1:1">
+      <c r="A120" s="45"/>
+    </row>
+    <row r="121" spans="1:1">
+      <c r="A121" s="45"/>
+    </row>
+    <row r="122" spans="1:1">
+      <c r="A122" s="45"/>
+    </row>
+    <row r="123" spans="1:1">
+      <c r="A123" s="45"/>
+    </row>
+    <row r="124" spans="1:1">
+      <c r="A124" s="45"/>
+    </row>
+    <row r="125" spans="1:1">
+      <c r="A125" s="45"/>
+    </row>
+    <row r="126" spans="1:1">
+      <c r="A126" s="45"/>
+    </row>
+    <row r="127" spans="1:1">
+      <c r="A127" s="45"/>
+    </row>
+    <row r="128" spans="1:1">
+      <c r="A128" s="45"/>
+    </row>
+    <row r="129" spans="1:1">
+      <c r="A129" s="45"/>
+    </row>
+    <row r="130" spans="1:1">
+      <c r="A130" s="45"/>
+    </row>
+    <row r="131" spans="1:1">
+      <c r="A131" s="45"/>
+    </row>
+    <row r="132" spans="1:1">
+      <c r="A132" s="45"/>
+    </row>
+    <row r="133" spans="1:1">
+      <c r="A133" s="45"/>
+    </row>
+    <row r="134" spans="1:1">
+      <c r="A134" s="45"/>
+    </row>
+    <row r="135" spans="1:1">
+      <c r="A135" s="45"/>
+    </row>
+    <row r="136" spans="1:1">
+      <c r="A136" s="45"/>
+    </row>
+    <row r="137" spans="1:1">
+      <c r="A137" s="45"/>
+    </row>
+    <row r="138" spans="1:1">
+      <c r="A138" s="45"/>
+    </row>
+    <row r="139" spans="1:1">
+      <c r="A139" s="45"/>
+    </row>
+    <row r="140" spans="1:1">
+      <c r="A140" s="45"/>
+    </row>
+    <row r="141" spans="1:1">
+      <c r="A141" s="45"/>
+    </row>
+    <row r="142" spans="1:1">
+      <c r="A142" s="45"/>
+    </row>
+    <row r="143" spans="1:1">
+      <c r="A143" s="45"/>
+    </row>
+    <row r="144" spans="1:1">
+      <c r="A144" s="45"/>
+    </row>
+    <row r="145" spans="1:1">
+      <c r="A145" s="45"/>
+    </row>
+    <row r="146" spans="1:1">
+      <c r="A146" s="45"/>
+    </row>
+    <row r="147" spans="1:1">
+      <c r="A147" s="45"/>
+    </row>
+    <row r="148" spans="1:1">
+      <c r="A148" s="45"/>
+    </row>
+    <row r="149" spans="1:1">
+      <c r="A149" s="45"/>
+    </row>
+    <row r="150" spans="1:1">
+      <c r="A150" s="45"/>
+    </row>
+    <row r="151" spans="1:1">
+      <c r="A151" s="45"/>
+    </row>
+    <row r="152" spans="1:1">
+      <c r="A152" s="45"/>
+    </row>
+    <row r="153" spans="1:1">
+      <c r="A153" s="45"/>
+    </row>
+    <row r="154" spans="1:1">
+      <c r="A154" s="45"/>
+    </row>
+    <row r="155" spans="1:1">
+      <c r="A155" s="45"/>
+    </row>
+    <row r="156" spans="1:1">
+      <c r="A156" s="45"/>
+    </row>
+    <row r="157" spans="1:1">
+      <c r="A157" s="45"/>
+    </row>
+    <row r="158" spans="1:1">
+      <c r="A158" s="45"/>
+    </row>
+    <row r="159" spans="1:1">
+      <c r="A159" s="45"/>
+    </row>
+    <row r="160" spans="1:1">
+      <c r="A160" s="45"/>
+    </row>
+    <row r="161" spans="1:1">
+      <c r="A161" s="45"/>
+    </row>
+    <row r="162" spans="1:1">
+      <c r="A162" s="45"/>
+    </row>
+    <row r="163" spans="1:1">
+      <c r="A163" s="45"/>
+    </row>
+    <row r="164" spans="1:1">
+      <c r="A164" s="45"/>
+    </row>
+    <row r="165" spans="1:1">
+      <c r="A165" s="45"/>
+    </row>
+    <row r="166" spans="1:1">
+      <c r="A166" s="45"/>
+    </row>
+    <row r="167" spans="1:1">
+      <c r="A167" s="45"/>
+    </row>
+    <row r="168" spans="1:1">
+      <c r="A168" s="45"/>
+    </row>
+    <row r="169" spans="1:1">
+      <c r="A169" s="45"/>
+    </row>
+    <row r="170" spans="1:1">
+      <c r="A170" s="45"/>
+    </row>
+    <row r="171" spans="1:1">
+      <c r="A171" s="45"/>
+    </row>
+    <row r="172" spans="1:1">
+      <c r="A172" s="45"/>
+    </row>
+    <row r="173" spans="1:1">
+      <c r="A173" s="45"/>
+    </row>
+    <row r="174" spans="1:1">
+      <c r="A174" s="45"/>
+    </row>
+    <row r="175" spans="1:1">
+      <c r="A175" s="45"/>
+    </row>
+    <row r="176" spans="1:1">
+      <c r="A176" s="45"/>
+    </row>
+    <row r="177" spans="1:1">
+      <c r="A177" s="45"/>
+    </row>
+    <row r="178" spans="1:1">
+      <c r="A178" s="45"/>
+    </row>
+    <row r="179" spans="1:1">
+      <c r="A179" s="45"/>
+    </row>
+    <row r="180" spans="1:1">
+      <c r="A180" s="45"/>
+    </row>
+    <row r="181" spans="1:1">
+      <c r="A181" s="45"/>
+    </row>
+    <row r="182" spans="1:1">
+      <c r="A182" s="45"/>
+    </row>
+    <row r="183" spans="1:1">
+      <c r="A183" s="45"/>
+    </row>
+    <row r="184" spans="1:1">
+      <c r="A184" s="45"/>
+    </row>
+    <row r="185" spans="1:1">
+      <c r="A185" s="45"/>
+    </row>
+    <row r="186" spans="1:1">
+      <c r="A186" s="45"/>
+    </row>
+    <row r="187" spans="1:1">
+      <c r="A187" s="45"/>
+    </row>
+    <row r="188" spans="1:1">
+      <c r="A188" s="45"/>
+    </row>
+    <row r="189" spans="1:1">
+      <c r="A189" s="45"/>
+    </row>
+    <row r="190" spans="1:1">
+      <c r="A190" s="45"/>
+    </row>
+    <row r="191" spans="1:1">
+      <c r="A191" s="45"/>
+    </row>
+    <row r="192" spans="1:1">
+      <c r="A192" s="45"/>
+    </row>
+    <row r="193" spans="1:1">
+      <c r="A193" s="45"/>
+    </row>
+    <row r="194" spans="1:1">
+      <c r="A194" s="45"/>
+    </row>
+    <row r="195" spans="1:1">
+      <c r="A195" s="45"/>
+    </row>
+    <row r="196" spans="1:1">
+      <c r="A196" s="45"/>
+    </row>
+    <row r="197" spans="1:1">
+      <c r="A197" s="45"/>
+    </row>
+    <row r="198" spans="1:1">
+      <c r="A198" s="45"/>
+    </row>
+    <row r="199" spans="1:1">
+      <c r="A199" s="45"/>
+    </row>
+    <row r="200" spans="1:1">
+      <c r="A200" s="45"/>
+    </row>
+    <row r="201" spans="1:1">
+      <c r="A201" s="45"/>
+    </row>
+    <row r="202" spans="1:1">
+      <c r="A202" s="45"/>
+    </row>
+    <row r="203" spans="1:1">
+      <c r="A203" s="45"/>
+    </row>
+    <row r="204" spans="1:1">
+      <c r="A204" s="45"/>
+    </row>
+    <row r="205" spans="1:1">
+      <c r="A205" s="45"/>
+    </row>
+    <row r="206" spans="1:1">
+      <c r="A206" s="45"/>
+    </row>
+    <row r="207" spans="1:1">
+      <c r="A207" s="45"/>
+    </row>
+    <row r="208" spans="1:1">
+      <c r="A208" s="45"/>
+    </row>
+    <row r="209" spans="1:1">
+      <c r="A209" s="45"/>
+    </row>
+    <row r="210" spans="1:1">
+      <c r="A210" s="45"/>
+    </row>
+    <row r="211" spans="1:1">
+      <c r="A211" s="45"/>
+    </row>
+    <row r="212" spans="1:1">
+      <c r="A212" s="45"/>
+    </row>
+    <row r="213" spans="1:1">
+      <c r="A213" s="45"/>
+    </row>
+    <row r="214" spans="1:1">
+      <c r="A214" s="45"/>
+    </row>
+    <row r="215" spans="1:1">
+      <c r="A215" s="45"/>
+    </row>
+    <row r="216" spans="1:1">
+      <c r="A216" s="45"/>
+    </row>
+    <row r="217" spans="1:1">
+      <c r="A217" s="45"/>
+    </row>
+    <row r="218" spans="1:1">
+      <c r="A218" s="45"/>
+    </row>
+    <row r="219" spans="1:1">
+      <c r="A219" s="45"/>
+    </row>
+    <row r="220" spans="1:1">
+      <c r="A220" s="45"/>
+    </row>
+    <row r="221" spans="1:1">
+      <c r="A221" s="45"/>
+    </row>
+    <row r="222" spans="1:1">
+      <c r="A222" s="45"/>
+    </row>
+    <row r="223" spans="1:1">
+      <c r="A223" s="45"/>
+    </row>
+    <row r="224" spans="1:1">
+      <c r="A224" s="45"/>
+    </row>
+    <row r="225" spans="1:1">
+      <c r="A225" s="45"/>
+    </row>
+    <row r="226" spans="1:1">
+      <c r="A226" s="45"/>
+    </row>
+    <row r="227" spans="1:1">
+      <c r="A227" s="45"/>
+    </row>
+    <row r="228" spans="1:1">
+      <c r="A228" s="45"/>
+    </row>
+    <row r="229" spans="1:1">
+      <c r="A229" s="45"/>
+    </row>
+    <row r="230" spans="1:1">
+      <c r="A230" s="45"/>
+    </row>
+    <row r="231" spans="1:1">
+      <c r="A231" s="45"/>
+    </row>
+    <row r="232" spans="1:1">
+      <c r="A232" s="45"/>
+    </row>
+    <row r="233" spans="1:1">
+      <c r="A233" s="45"/>
+    </row>
+    <row r="234" spans="1:1">
+      <c r="A234" s="45"/>
+    </row>
+    <row r="235" spans="1:1">
+      <c r="A235" s="45"/>
+    </row>
+    <row r="236" spans="1:1">
+      <c r="A236" s="45"/>
+    </row>
+    <row r="237" spans="1:1">
+      <c r="A237" s="45"/>
+    </row>
+    <row r="238" spans="1:1">
+      <c r="A238" s="45"/>
+    </row>
+    <row r="239" spans="1:1">
+      <c r="A239" s="45"/>
+    </row>
+    <row r="240" spans="1:1">
+      <c r="A240" s="45"/>
+    </row>
+    <row r="241" spans="1:1">
+      <c r="A241" s="45"/>
+    </row>
+    <row r="242" spans="1:1">
+      <c r="A242" s="45"/>
+    </row>
+    <row r="243" spans="1:1">
+      <c r="A243" s="45"/>
+    </row>
+    <row r="244" spans="1:1">
+      <c r="A244" s="45"/>
+    </row>
+    <row r="245" spans="1:1">
+      <c r="A245" s="45"/>
+    </row>
+    <row r="246" spans="1:1">
+      <c r="A246" s="45"/>
+    </row>
+    <row r="247" spans="1:1">
+      <c r="A247" s="45"/>
+    </row>
+    <row r="248" spans="1:1">
+      <c r="A248" s="45"/>
+    </row>
+    <row r="249" spans="1:1">
+      <c r="A249" s="45"/>
+    </row>
+    <row r="250" spans="1:1">
+      <c r="A250" s="45"/>
+    </row>
+    <row r="251" spans="1:1">
+      <c r="A251" s="45"/>
+    </row>
+    <row r="252" spans="1:1">
+      <c r="A252" s="45"/>
+    </row>
+    <row r="253" spans="1:1">
+      <c r="A253" s="45"/>
+    </row>
+    <row r="254" spans="1:1">
+      <c r="A254" s="45"/>
+    </row>
+    <row r="255" spans="1:1">
+      <c r="A255" s="45"/>
+    </row>
+    <row r="256" spans="1:1">
+      <c r="A256" s="45"/>
+    </row>
+    <row r="257" spans="1:1">
+      <c r="A257" s="45"/>
+    </row>
+    <row r="258" spans="1:1">
+      <c r="A258" s="45"/>
+    </row>
+    <row r="259" spans="1:1">
+      <c r="A259" s="45"/>
+    </row>
+    <row r="260" spans="1:1">
+      <c r="A260" s="45"/>
+    </row>
+    <row r="261" spans="1:1">
+      <c r="A261" s="45"/>
+    </row>
+    <row r="262" spans="1:1">
+      <c r="A262" s="45"/>
+    </row>
+    <row r="263" spans="1:1">
+      <c r="A263" s="45"/>
+    </row>
+    <row r="264" spans="1:1">
+      <c r="A264" s="45"/>
+    </row>
+    <row r="265" spans="1:1">
+      <c r="A265" s="45"/>
+    </row>
+    <row r="266" spans="1:1">
+      <c r="A266" s="45"/>
+    </row>
+    <row r="267" spans="1:1">
+      <c r="A267" s="45"/>
+    </row>
+    <row r="268" spans="1:1">
+      <c r="A268" s="45"/>
+    </row>
+    <row r="269" spans="1:1">
+      <c r="A269" s="45"/>
+    </row>
+    <row r="270" spans="1:1">
+      <c r="A270" s="45"/>
+    </row>
+    <row r="271" spans="1:1">
+      <c r="A271" s="45"/>
+    </row>
+    <row r="272" spans="1:1">
+      <c r="A272" s="45"/>
+    </row>
+    <row r="273" spans="1:1">
+      <c r="A273" s="45"/>
+    </row>
+    <row r="274" spans="1:1">
+      <c r="A274" s="45"/>
+    </row>
+    <row r="275" spans="1:1">
+      <c r="A275" s="45"/>
+    </row>
+    <row r="276" spans="1:1">
+      <c r="A276" s="45"/>
+    </row>
+    <row r="277" spans="1:1">
+      <c r="A277" s="45"/>
+    </row>
+    <row r="278" spans="1:1">
+      <c r="A278" s="45"/>
+    </row>
+    <row r="279" spans="1:1">
+      <c r="A279" s="45"/>
+    </row>
+    <row r="280" spans="1:1">
+      <c r="A280" s="45"/>
+    </row>
+    <row r="281" spans="1:1">
+      <c r="A281" s="45"/>
+    </row>
+    <row r="282" spans="1:1">
+      <c r="A282" s="45"/>
+    </row>
+    <row r="283" spans="1:1">
+      <c r="A283" s="45"/>
+    </row>
+    <row r="284" spans="1:1">
+      <c r="A284" s="45"/>
+    </row>
+    <row r="285" spans="1:1">
+      <c r="A285" s="45"/>
+    </row>
+    <row r="286" spans="1:1">
+      <c r="A286" s="45"/>
+    </row>
+    <row r="287" spans="1:1">
+      <c r="A287" s="45"/>
+    </row>
+    <row r="288" spans="1:1">
+      <c r="A288" s="45"/>
+    </row>
+    <row r="289" spans="1:1">
+      <c r="A289" s="45"/>
+    </row>
+    <row r="290" spans="1:1">
+      <c r="A290" s="45"/>
+    </row>
+    <row r="291" spans="1:1">
+      <c r="A291" s="45"/>
+    </row>
+    <row r="292" spans="1:1">
+      <c r="A292" s="45"/>
+    </row>
+    <row r="293" spans="1:1">
+      <c r="A293" s="45"/>
+    </row>
+    <row r="294" spans="1:1">
+      <c r="A294" s="45"/>
+    </row>
+    <row r="295" spans="1:1">
+      <c r="A295" s="45"/>
+    </row>
+    <row r="296" spans="1:1">
+      <c r="A296" s="45"/>
+    </row>
+    <row r="297" spans="1:1">
+      <c r="A297" s="45"/>
+    </row>
+    <row r="298" spans="1:1">
+      <c r="A298" s="45"/>
+    </row>
+    <row r="299" spans="1:1">
+      <c r="A299" s="45"/>
+    </row>
+    <row r="300" spans="1:1">
+      <c r="A300" s="45"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1436,19 +2317,21 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="10.85546875" customWidth="1"/>
+    <col min="3" max="3" width="9.85546875" style="34" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.7109375" style="34" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="14.7109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17" customWidth="1"/>
     <col min="12" max="12" width="10.5703125" customWidth="1"/>
     <col min="13" max="13" width="10.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="27" customHeight="1">
       <c r="B1" s="32" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="10.5" customHeight="1"/>
@@ -1472,7 +2355,7 @@
         <v>17</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H3" s="6" t="s">
         <v>26</v>
@@ -1481,148 +2364,260 @@
         <v>31</v>
       </c>
       <c r="J3" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="K3" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="K3" s="6" t="s">
+      <c r="L3" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="L3" s="6" t="s">
+      <c r="M3" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="M3" s="6" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
+    </row>
+    <row r="4" spans="1:13" ht="60">
       <c r="A4" s="4"/>
       <c r="B4" s="42">
         <v>46301</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E4" t="s">
-        <v>45</v>
-      </c>
-      <c r="F4" t="s">
-        <v>24</v>
-      </c>
-      <c r="H4" t="s">
-        <v>27</v>
-      </c>
-      <c r="I4" t="s">
+      <c r="E4" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" s="1">
+        <v>10</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="I4" s="1" t="s">
         <v>32</v>
       </c>
+      <c r="J4" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="4"/>
       <c r="B5" s="42">
         <v>46301</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D5" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="E5" t="s">
-        <v>114</v>
-      </c>
+      <c r="E5" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G5" s="1">
+        <v>10</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="4"/>
       <c r="B6" s="42">
         <v>46301</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E6" t="s">
-        <v>115</v>
-      </c>
+      <c r="E6" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G6" s="1">
+        <v>10</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="4"/>
       <c r="B7" s="42">
         <v>46301</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E7" t="s">
-        <v>116</v>
-      </c>
+      <c r="E7" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G7" s="1">
+        <v>10</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" s="4"/>
       <c r="B8" s="42">
         <v>46301</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E8" t="s">
-        <v>117</v>
-      </c>
+      <c r="E8" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="4"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="1"/>
+      <c r="B9" s="42">
+        <v>46301</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" t="s">
+        <v>116</v>
+      </c>
+      <c r="F9" t="s">
+        <v>25</v>
+      </c>
+      <c r="G9" s="1">
+        <v>25</v>
+      </c>
+      <c r="H9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I9" t="s">
+        <v>33</v>
+      </c>
+      <c r="J9" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="10" spans="1:13">
       <c r="A10" s="4"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="1"/>
+      <c r="B10" s="42">
+        <v>46301</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" t="s">
+        <v>118</v>
+      </c>
+      <c r="F10" t="s">
+        <v>24</v>
+      </c>
+      <c r="G10" s="1">
+        <v>15</v>
+      </c>
+      <c r="H10" t="s">
+        <v>29</v>
+      </c>
+      <c r="I10" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="11" spans="1:13">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
+      <c r="C11" s="1"/>
       <c r="D11" s="1"/>
     </row>
     <row r="12" spans="1:13">
       <c r="A12" s="4"/>
       <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
+      <c r="C12" s="1"/>
       <c r="D12" s="1"/>
     </row>
     <row r="13" spans="1:13">
       <c r="A13" s="4"/>
       <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
+      <c r="C13" s="1"/>
       <c r="D13" s="1"/>
     </row>
     <row r="14" spans="1:13">
       <c r="A14" s="4"/>
       <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
+      <c r="C14" s="1"/>
       <c r="D14" s="1"/>
     </row>
     <row r="15" spans="1:13">
       <c r="A15" s="4"/>
       <c r="B15" s="4"/>
-      <c r="C15" s="4"/>
+      <c r="C15" s="1"/>
       <c r="D15" s="43"/>
     </row>
     <row r="16" spans="1:13">
       <c r="A16" s="4"/>
       <c r="B16" s="4"/>
-      <c r="C16" s="4"/>
+      <c r="C16" s="1"/>
       <c r="D16" s="43"/>
     </row>
   </sheetData>
@@ -1691,7 +2686,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="18.75" thickBot="1">
       <c r="A1" s="32" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="36" customFormat="1" ht="15.75">
@@ -1699,16 +2694,16 @@
         <v>11</v>
       </c>
       <c r="B2" s="41" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C2" s="41" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D2" s="41" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="15.75">
@@ -1721,15 +2716,15 @@
       </c>
       <c r="C3" s="38">
         <f>COUNTIFS(Problems!C:C,A3,Problems!H:H,"✅ Done")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D3" s="21">
         <f>IF(B3=0,0,C3/B3)</f>
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="E3" s="11">
         <f>SUMIF(Problems!C:C,A3,Problems!G:G)</f>
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="15.75">
@@ -1738,19 +2733,19 @@
       </c>
       <c r="B4" s="38">
         <f>COUNTIF(Problems!C:C,A4)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C4" s="38">
         <f>COUNTIFS(Problems!C:C,A4,Problems!H:H,"✅ Done")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D4" s="21">
         <f>IF(B4=0,0,C4/B4)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" s="11">
         <f>SUMIF(Problems!C:C,A4,Problems!G:G)</f>
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="15.75">
@@ -1759,19 +2754,19 @@
       </c>
       <c r="B5" s="38">
         <f>COUNTIF(Problems!C:C,A5)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C5" s="38">
         <f>COUNTIFS(Problems!C:C,A5,Problems!H:H,"✅ Done")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D5" s="21">
         <f t="shared" ref="D5:D13" si="0">IF(B5=0,0,C5/B5)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" s="11">
         <f>SUMIF(Problems!C:C,A5,Problems!G:G)</f>
-        <v>0</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="15.75">
@@ -1959,7 +2954,7 @@
   <sheetData>
     <row r="1" spans="1:2" ht="26.25" customHeight="1">
       <c r="A1" s="32" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -1972,89 +2967,89 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>78</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>80</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>82</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>84</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="20" spans="1:1">
       <c r="A20" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="23" spans="1:1">
       <c r="A23" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="24" spans="1:1">
       <c r="A24" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -2072,7 +3067,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="24" customHeight="1">
       <c r="A1" s="32" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" spans="1:7" s="36" customFormat="1" ht="15.75">
@@ -2083,16 +3078,16 @@
         <v>11</v>
       </c>
       <c r="C2" s="35" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D2" s="35" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E2" s="35" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F2" s="35" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G2" s="35" t="s">
         <v>26</v>
@@ -2134,7 +3129,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C10" s="4"/>
     </row>
@@ -2146,19 +3141,19 @@
         <v>3</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F11" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="G11" s="4" t="s">
         <v>103</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -2179,7 +3174,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="25.5" customHeight="1">
       <c r="B1" s="32" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3" spans="1:6">

</xml_diff>